<commit_message>
added more test cases
</commit_message>
<xml_diff>
--- a/TCs.xlsx
+++ b/TCs.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="126">
   <si>
     <t xml:space="preserve">TC ID :</t>
   </si>
@@ -115,6 +115,39 @@
   </si>
   <si>
     <t xml:space="preserve">fail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_HOME_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test “start order” button is rendered when enter a valid name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the browser
+2. navigate to home page URL
+3. enter a valid name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“start order” button should be rendered on the the first letter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_HOME_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify valid name and Start ordering navigate to menu page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the browser
+2. navigate to home page URL
+3. enter a valid name
+4. click the "Start ordering" button. 
+5. observe the next page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is navigated from the home page to the menu page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ensures that entering a valid name and clicking "Start ordering" successfully transitions the user from the home page to the menu page.</t>
   </si>
   <si>
     <t xml:space="preserve">TC_MENU_001</t>
@@ -189,6 +222,52 @@
     <t xml:space="preserve">Verifies that adding a pizza from the menu correctly updates the cart item count shown in the UI.</t>
   </si>
   <si>
+    <t xml:space="preserve">TC_MENU_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify "Add to cart" button is not displayed for sold-out pizzas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- User can navigate to the menu page from the home page.
+- At least one pizza is marked as "Sold out" on the menu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the home page.
+2. Enter a valid name and click "Start ordering" to go to the menu page.
+3. On the menu page, locate a pizza item that is marked as "Sold out".
+4. Check the button displayed for this sold-out pizza item.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The "Add to cart" button is NOT displayed for sold-out pizza items.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ensures that pizzas marked as sold out are not orderable and do not show an "Add to cart" button.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_MENU_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify navigating to cart page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- User can navigate to the menu page from the home page.
+- At least one pizza is available (not sold out) on the menu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the home page.
+2. Enter a valid name and click "Start ordering" to go to the menu page.
+3. On the menu page, locate the first available pizza.
+4. Click the "Add to cart" button for that pizza.
+5. Click the "Open cart" button in the footer to navigate to the cart page.
+6. Observe the number of items shown in the cart.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is navigated to the cart page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verifies that adding a pizza from the menu and opening the cart correctly navigates to the cart page and shows one cart item.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC_CART_001</t>
   </si>
   <si>
@@ -264,6 +343,55 @@
   </si>
   <si>
     <t xml:space="preserve">Ensures that it is correctly clears the cart and displays an appropriate empty state to the user.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_CART_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify decreasing item quantity updates quantity and total correctly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Cart contains a single pizza with quantity = 2 or more.
+- User is on the cart page with "-" (decrease) button available.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Ensure the pizza in the cart has quantity = 2
+2. Note the current cart total (TotalBefore).
+3. Click the "-" (decrease quantity) button once for that pizza.
+4. Read the updated quantity.
+5. Read the updated cart total (TotalAfter).
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantity decreases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verifies that the "-" control correctly reduces the quantity of a cart item
+and that the cart total is updated to reflect the change.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_CART_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify user cannot proceed to order when cart is empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- User is on the cart page.
+- Cart contains no items</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the cart page.
+2. If there are any items, use "Clear cart" to remove them all.
+3. Observe the "Order pizzas" (or equivalent) button/link.
+4. Try to click "Order pizzas" when the cart is empty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is not allowed to proceed to the order page with an empty cart.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ensures that the user cannot start the checkout flow with an empty cart,
+enforcing a proper business rule.</t>
   </si>
   <si>
     <t xml:space="preserve">TC_ORDER_001</t>
@@ -486,14 +614,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF111111"/>
-        <bgColor rgb="FF000000"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <fgColor rgb="FF111111"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -538,7 +666,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -571,6 +699,18 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -583,16 +723,8 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -855,7 +987,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.22"/>
@@ -913,309 +1045,454 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+    <row r="5" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+    <row r="8" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>26</v>
       </c>
     </row>
+    <row r="9" customFormat="false" ht="17.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="17.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="10"/>
+      <c r="G11" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="17.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="17.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="B14" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G11" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" s="11" customFormat="true" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
+      <c r="C14" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="F14" s="10" t="s">
         <v>35</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>38</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+    <row r="15" customFormat="false" ht="17.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="17.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="E17" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="F17" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="G17" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" s="14" customFormat="true" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="B20" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="C20" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="G17" s="12" t="s">
+      <c r="D20" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="G20" s="11" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="8" t="s">
+    <row r="23" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="B23" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="C23" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="G20" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
+      <c r="D23" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="E23" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="F23" s="8" t="s">
         <v>53</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>56</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="120.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="E26" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="F26" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="G26" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="B29" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="C29" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="G26" s="14" t="s">
+      <c r="D29" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="G29" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="150.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="D29" s="12" t="s">
+    <row r="32" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="E29" s="12" t="s">
+      <c r="B32" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="F29" s="12" t="s">
+      <c r="C32" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="G29" s="12" t="s">
+      <c r="D32" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="G32" s="11" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="C32" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="D32" s="12" t="s">
+    <row r="35" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E32" s="12" t="s">
+      <c r="B35" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="F32" s="12" t="s">
+      <c r="C35" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="G32" s="12" t="s">
+      <c r="D35" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="G35" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="120.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="G38" s="15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="G41" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="150.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="G47" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="G50" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="150.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="D35" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="E35" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="F35" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="G35" s="12" t="s">
+    <row r="53" customFormat="false" ht="150.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="F53" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="G53" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B38" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="C38" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="D38" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="E38" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="G38" s="12" t="s">
+    <row r="56" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G56" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B41" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="C41" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="D41" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="E41" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="F41" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="G41" s="12" t="s">
+    <row r="59" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D59" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F59" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="G59" s="8" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G1:G1017" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G1:G1035" type="list">
       <formula1>"blocked,pass,fail,pending"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1228,7 +1505,7 @@
     <oddFooter/>
   </headerFooter>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="13" man="true" max="16383" min="0"/>
+    <brk id="19" man="true" max="16383" min="0"/>
   </rowBreaks>
 </worksheet>
 </file>

</xml_diff>